<commit_message>
KrakenBoss AI 행동 마무리 #67
 - UtilityAI 편리 사용을 위한 Function Preset 제작
 - Action이 시작과 동시에 끊기는 것을 방지하기 위한 구조 변경
 - AttackAction을 한 후에 일정 시간동안 나오지 않도록 CanAttack Axis 수정
 - Action의 최소, 최대 Distance 설정을 할 수 있게 수정
 - AgeTime, CoolTime, AgeRate를 UtilityAIData에서 한번에 수정할 수 있게 변경
 - Kraken의 최종 UtilityAI Data 변수 세팅 및 테스트
</commit_message>
<xml_diff>
--- a/GameDatas/AttributeSet/AttributeExcel.xlsx
+++ b/GameDatas/AttributeSet/AttributeExcel.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="Polaris Office Sheet" lastEdited="4" lowestEdited="4" rupBuild="10.105.305.56234"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="AttributeData" sheetId="1" r:id="rId1"/>
@@ -1815,7 +1815,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="0">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="D6" s="0">
         <v>0</v>
@@ -1836,7 +1836,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="0">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="D7" s="0">
         <v>0</v>
@@ -1857,7 +1857,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="0">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="D8" s="0">
         <v>0</v>

</xml_diff>